<commit_message>
malsim khanepani estimate complete
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/malsim khanepaani/malsim khanepaani.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/malsim khanepaani/malsim khanepaani.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB3E3914-8EEC-4F35-AD86-2BCAB2B3FE10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
@@ -39,7 +40,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$41</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -173,30 +174,6 @@
     <t>-for pipe laying</t>
   </si>
   <si>
-    <r>
-      <t>Earthwork in Excavation in ordinary soil (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Preeti"/>
-      </rPr>
-      <t>vGg] k'g{] sfo{</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
     <t>-from source1 to tank 3, 32mm dia pipe</t>
   </si>
   <si>
@@ -239,16 +216,38 @@
       <t>dnl;d vfg]kfgL</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t>Earthwork in Excavation in ordinary soil (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <rFont val="Preeti"/>
+      </rPr>
+      <t>vGg] k'g{] sfo{</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -321,44 +320,15 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Preeti"/>
     </font>
     <font>
-      <b/>
       <sz val="14"/>
-      <color rgb="FFFF0000"/>
       <name val="Preeti"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Preeti"/>
-    </font>
-    <font>
       <sz val="14"/>
       <name val="Preeti"/>
     </font>
@@ -432,13 +402,13 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -446,7 +416,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -470,14 +440,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -496,7 +466,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -511,7 +481,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -533,41 +503,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -588,32 +543,26 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3"/>
+    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
-    <cellStyle name="Normal 3" xfId="5"/>
-    <cellStyle name="Percent 2" xfId="4"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -629,7 +578,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -723,7 +672,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -782,7 +731,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -846,9 +795,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -886,9 +835,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -923,7 +872,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -958,7 +907,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1131,135 +1080,135 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S41"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="19"/>
+    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" style="19" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="9.109375" style="19"/>
+    <col min="9" max="9" width="9.5703125" style="19" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" style="19"/>
     <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="19"/>
+    <col min="17" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-    </row>
-    <row r="2" spans="1:19" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="62" t="s">
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+    </row>
+    <row r="2" spans="1:19" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="63" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A4" s="63" t="s">
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
+      <c r="J3" s="43"/>
+      <c r="K3" s="43"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
-    </row>
-    <row r="5" spans="1:19" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="64" t="s">
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
+      <c r="I4" s="43"/>
+      <c r="J4" s="43"/>
+      <c r="K4" s="43"/>
+    </row>
+    <row r="5" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="64"/>
-      <c r="K5" s="64"/>
-    </row>
-    <row r="6" spans="1:19" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A6" s="59" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="59"/>
-      <c r="C6" s="59"/>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
-      <c r="F6" s="59"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+    </row>
+    <row r="6" spans="1:19" ht="18" x14ac:dyDescent="0.25">
+      <c r="A6" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="60" t="s">
+      <c r="H6" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="60"/>
-      <c r="J6" s="60"/>
-      <c r="K6" s="60"/>
-    </row>
-    <row r="7" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="54" t="s">
+      <c r="I6" s="40"/>
+      <c r="J6" s="40"/>
+      <c r="K6" s="40"/>
+    </row>
+    <row r="7" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="55" t="s">
+      <c r="H7" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="I7" s="55"/>
-      <c r="J7" s="55"/>
-      <c r="K7" s="55"/>
-    </row>
-    <row r="8" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
+      <c r="K7" s="48"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
@@ -1294,99 +1243,99 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" ht="33" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
         <v>1</v>
       </c>
-      <c r="B9" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="39"/>
-      <c r="H9" s="39"/>
-      <c r="I9" s="39"/>
-      <c r="J9" s="40"/>
+      <c r="B9" s="52" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="18"/>
       <c r="K9" s="17"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="39">
+      <c r="C10" s="17">
         <v>1</v>
       </c>
-      <c r="D10" s="42">
+      <c r="D10" s="33">
         <v>175</v>
       </c>
-      <c r="E10" s="39">
+      <c r="E10" s="17">
         <v>0.3</v>
       </c>
-      <c r="F10" s="39">
+      <c r="F10" s="17">
         <v>0.45</v>
       </c>
-      <c r="G10" s="42">
+      <c r="G10" s="33">
         <f t="shared" ref="G10:G12" si="0">PRODUCT(C10:F10)</f>
         <v>23.625</v>
       </c>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39"/>
-      <c r="J10" s="40"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="18"/>
       <c r="K10" s="17"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
-      <c r="B11" s="41"/>
-      <c r="C11" s="39">
+      <c r="B11" s="32"/>
+      <c r="C11" s="17">
         <v>1</v>
       </c>
-      <c r="D11" s="42">
+      <c r="D11" s="33">
         <v>150</v>
       </c>
-      <c r="E11" s="39">
+      <c r="E11" s="17">
         <v>0.3</v>
       </c>
-      <c r="F11" s="39">
+      <c r="F11" s="17">
         <v>0.45</v>
       </c>
-      <c r="G11" s="42">
+      <c r="G11" s="33">
         <f t="shared" si="0"/>
         <v>20.25</v>
       </c>
-      <c r="H11" s="39"/>
-      <c r="I11" s="39"/>
-      <c r="J11" s="40"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="18"/>
       <c r="K11" s="17"/>
       <c r="R11" s="19">
         <f>480/3.281</f>
         <v>146.29686071319719</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
-      <c r="B12" s="41"/>
-      <c r="C12" s="39">
+      <c r="B12" s="32"/>
+      <c r="C12" s="17">
         <v>1</v>
       </c>
-      <c r="D12" s="42">
-        <v>400</v>
-      </c>
-      <c r="E12" s="39">
+      <c r="D12" s="33">
+        <v>415</v>
+      </c>
+      <c r="E12" s="17">
         <v>0.3</v>
       </c>
-      <c r="F12" s="39">
+      <c r="F12" s="17">
         <v>0.45</v>
       </c>
-      <c r="G12" s="42">
+      <c r="G12" s="33">
         <f t="shared" si="0"/>
-        <v>54</v>
-      </c>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="40"/>
+        <v>56.024999999999999</v>
+      </c>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="18"/>
       <c r="K12" s="17"/>
       <c r="R12" s="19">
         <f>160+135+301</f>
@@ -1397,28 +1346,28 @@
         <v>181.65193538555317</v>
       </c>
     </row>
-    <row r="13" spans="1:19" s="35" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="43" t="s">
+      <c r="B13" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="46"/>
-      <c r="F13" s="46"/>
-      <c r="G13" s="47">
+      <c r="C13" s="3"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="54">
         <f>SUM(G10:G12)</f>
-        <v>97.875</v>
-      </c>
-      <c r="H13" s="48" t="s">
+        <v>99.9</v>
+      </c>
+      <c r="H13" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="I13" s="49">
+      <c r="I13" s="6">
         <v>963.05</v>
       </c>
-      <c r="J13" s="47">
+      <c r="J13" s="54">
         <f>G13*I13</f>
-        <v>94258.518749999988</v>
+        <v>96208.695000000007</v>
       </c>
       <c r="K13" s="5"/>
       <c r="R13" s="35">
@@ -1429,7 +1378,7 @@
         <v>386.77232551051509</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="32"/>
       <c r="C14" s="17"/>
@@ -1442,12 +1391,12 @@
       <c r="J14" s="18"/>
       <c r="K14" s="17"/>
     </row>
-    <row r="15" spans="1:19" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="16">
         <v>2</v>
       </c>
-      <c r="B15" s="38" t="s">
-        <v>42</v>
+      <c r="B15" s="52" t="s">
+        <v>41</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
@@ -1459,58 +1408,58 @@
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="16"/>
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="39">
+      <c r="C16" s="17">
         <v>1</v>
       </c>
-      <c r="D16" s="42">
+      <c r="D16" s="33">
         <f>SUM(D20:D22)-100</f>
         <v>1900</v>
       </c>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="42">
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="33">
         <f t="shared" ref="G16" si="1">PRODUCT(C16:F16)</f>
         <v>1900</v>
       </c>
-      <c r="H16" s="39"/>
-      <c r="I16" s="39"/>
-      <c r="J16" s="40"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="18"/>
       <c r="K16" s="17"/>
     </row>
-    <row r="17" spans="1:17" s="35" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="43" t="s">
+      <c r="B17" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="44"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
-      <c r="G17" s="47">
+      <c r="C17" s="3"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="54">
         <f>SUM(G16:G16)</f>
         <v>1900</v>
       </c>
-      <c r="H17" s="48" t="s">
-        <v>43</v>
-      </c>
-      <c r="I17" s="49">
+      <c r="H17" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I17" s="6">
         <f>5319.5/1000</f>
         <v>5.3194999999999997</v>
       </c>
-      <c r="J17" s="47">
+      <c r="J17" s="54">
         <f>G17*I17</f>
         <v>10107.049999999999</v>
       </c>
       <c r="K17" s="5"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="16"/>
-      <c r="B18" s="38"/>
+      <c r="B18" s="52"/>
       <c r="C18" s="17"/>
       <c r="D18" s="17"/>
       <c r="E18" s="17"/>
@@ -1521,7 +1470,7 @@
       <c r="J18" s="17"/>
       <c r="K18" s="17"/>
     </row>
-    <row r="19" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="16">
         <v>3</v>
       </c>
@@ -1544,10 +1493,10 @@
       <c r="J19" s="18"/>
       <c r="K19" s="17"/>
     </row>
-    <row r="20" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="16"/>
-      <c r="B20" s="50" t="s">
-        <v>39</v>
+      <c r="B20" s="38" t="s">
+        <v>38</v>
       </c>
       <c r="C20" s="17">
         <v>1</v>
@@ -1575,10 +1524,10 @@
         <v>97.006</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
-      <c r="B21" s="50" t="s">
-        <v>40</v>
+      <c r="B21" s="38" t="s">
+        <v>39</v>
       </c>
       <c r="C21" s="17">
         <v>1</v>
@@ -1602,10 +1551,10 @@
       <c r="J21" s="18"/>
       <c r="K21" s="17"/>
     </row>
-    <row r="22" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
-      <c r="B22" s="50" t="s">
-        <v>41</v>
+      <c r="B22" s="38" t="s">
+        <v>40</v>
       </c>
       <c r="C22" s="17">
         <v>1</v>
@@ -1629,7 +1578,7 @@
       <c r="J22" s="18"/>
       <c r="K22" s="17"/>
     </row>
-    <row r="23" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="34" t="s">
         <v>16</v>
@@ -1658,7 +1607,7 @@
         <v>324.30999999999995</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="32" t="s">
         <v>36</v>
@@ -1676,7 +1625,7 @@
       </c>
       <c r="K24" s="17"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -1689,12 +1638,12 @@
       <c r="J25" s="17"/>
       <c r="K25" s="17"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="16">
         <v>4</v>
       </c>
-      <c r="B26" s="38" t="s">
-        <v>44</v>
+      <c r="B26" s="52" t="s">
+        <v>43</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -1706,56 +1655,56 @@
       <c r="J26" s="17"/>
       <c r="K26" s="17"/>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
-      <c r="B27" s="41" t="s">
+      <c r="B27" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="39">
+      <c r="C27" s="17">
         <v>1</v>
       </c>
-      <c r="D27" s="42">
+      <c r="D27" s="33">
         <v>6</v>
       </c>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="42">
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="33">
         <f t="shared" ref="G27" si="4">PRODUCT(C27:F27)</f>
         <v>6</v>
       </c>
-      <c r="H27" s="39"/>
-      <c r="I27" s="39"/>
-      <c r="J27" s="40"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="18"/>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:17" s="35" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="43" t="s">
+      <c r="B28" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="44"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="46"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="47">
+      <c r="C28" s="3"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="54">
         <f>SUM(G27:G27)</f>
         <v>6</v>
       </c>
-      <c r="H28" s="48" t="s">
-        <v>43</v>
-      </c>
-      <c r="I28" s="49">
+      <c r="H28" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I28" s="6">
         <v>452</v>
       </c>
-      <c r="J28" s="47">
+      <c r="J28" s="54">
         <f>G28*I28</f>
         <v>2712</v>
       </c>
       <c r="K28" s="5"/>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="16"/>
-      <c r="B29" s="38"/>
+      <c r="B29" s="52"/>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
       <c r="E29" s="17"/>
@@ -1766,38 +1715,38 @@
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
     </row>
-    <row r="30" spans="1:17" s="35" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" s="35" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>5</v>
       </c>
-      <c r="B30" s="51" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" s="44">
+      <c r="B30" s="55" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="3">
         <v>1</v>
       </c>
-      <c r="D30" s="45"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="47">
+      <c r="D30" s="4"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="54">
         <f t="shared" ref="G30" si="5">PRODUCT(C30:F30)</f>
         <v>1</v>
       </c>
-      <c r="H30" s="48" t="s">
-        <v>46</v>
-      </c>
-      <c r="I30" s="49">
+      <c r="H30" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I30" s="6">
         <v>7000</v>
       </c>
-      <c r="J30" s="47">
+      <c r="J30" s="54">
         <f>G30*I30</f>
         <v>7000</v>
       </c>
       <c r="K30" s="5"/>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
-      <c r="B31" s="38"/>
+      <c r="B31" s="52"/>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
       <c r="E31" s="17"/>
@@ -1808,7 +1757,7 @@
       <c r="J31" s="17"/>
       <c r="K31" s="17"/>
     </row>
-    <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>6</v>
       </c>
@@ -1837,7 +1786,7 @@
       </c>
       <c r="K32" s="5"/>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="8"/>
       <c r="C33" s="3"/>
@@ -1850,7 +1799,7 @@
       <c r="J33" s="18"/>
       <c r="K33" s="5"/>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="21"/>
       <c r="B34" s="22" t="s">
         <v>20</v>
@@ -1864,11 +1813,11 @@
       <c r="I34" s="18"/>
       <c r="J34" s="18">
         <f>SUM(J9:J32)</f>
-        <v>333811.12874999997</v>
+        <v>335761.30499999999</v>
       </c>
       <c r="K34" s="25"/>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="M35" s="20"/>
       <c r="N35" s="20"/>
       <c r="O35" s="20"/>
@@ -1877,16 +1826,16 @@
       <c r="R35" s="20"/>
       <c r="S35" s="20"/>
     </row>
-    <row r="36" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="26"/>
       <c r="B36" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="52">
+      <c r="C36" s="45">
         <f>J34</f>
-        <v>333811.12874999997</v>
-      </c>
-      <c r="D36" s="53"/>
+        <v>335761.30499999999</v>
+      </c>
+      <c r="D36" s="46"/>
       <c r="E36" s="9">
         <v>100</v>
       </c>
@@ -1904,79 +1853,72 @@
       <c r="R36" s="19"/>
       <c r="S36" s="19"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B37" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="56">
+      <c r="C37" s="49">
         <v>300000</v>
       </c>
-      <c r="D37" s="57"/>
+      <c r="D37" s="50"/>
       <c r="E37" s="9"/>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B38" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C38" s="56">
+      <c r="C38" s="49">
         <f>C37-C40-C41</f>
         <v>285000</v>
       </c>
-      <c r="D38" s="57"/>
+      <c r="D38" s="50"/>
       <c r="E38" s="9">
         <f>C38/C36*100</f>
-        <v>85.377620892155477</v>
-      </c>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+        <v>84.881728703073762</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B39" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C39" s="58">
+      <c r="C39" s="51">
         <f>C36-C38</f>
-        <v>48811.128749999974</v>
-      </c>
-      <c r="D39" s="58"/>
+        <v>50761.304999999993</v>
+      </c>
+      <c r="D39" s="51"/>
       <c r="E39" s="9">
         <f>100-E38</f>
-        <v>14.622379107844523</v>
-      </c>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+        <v>15.118271296926238</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B40" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C40" s="52">
+      <c r="C40" s="45">
         <f>C37*0.03</f>
         <v>9000</v>
       </c>
-      <c r="D40" s="53"/>
+      <c r="D40" s="46"/>
       <c r="E40" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B41" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C41" s="52">
+      <c r="C41" s="45">
         <f>C37*0.02</f>
         <v>6000</v>
       </c>
-      <c r="D41" s="53"/>
+      <c r="D41" s="46"/>
       <c r="E41" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="C41:D41"/>
     <mergeCell ref="A7:F7"/>
@@ -1985,6 +1927,13 @@
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="C39:D39"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>

</xml_diff>